<commit_message>
remving temp files and adding filetype to .gitignore file
</commit_message>
<xml_diff>
--- a/NetLabz_Project_Checklist.xlsx
+++ b/NetLabz_Project_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NetLabz_Enterprise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3177AD8-8A2A-452F-85A3-501AEB8EAB05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6FE6765-2FFE-44C5-A5DE-8E720BA083D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="29692" windowHeight="11829" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="14915" windowHeight="11709" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1871" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1872" uniqueCount="933">
   <si>
     <t>Overall Progress</t>
   </si>
@@ -2833,6 +2833,9 @@
   </si>
   <si>
     <t>NetLabz Enterprise  — Project Tracker</t>
+  </si>
+  <si>
+    <t>Used AI to list file types that are common with VM's so as not to miss any, creating vulnerability.</t>
   </si>
 </sst>
 </file>
@@ -3658,7 +3661,7 @@
       </c>
       <c r="B4" s="4">
         <f>IF(B5=0,0,B6/B5)</f>
-        <v>0</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>1</v>
@@ -3688,7 +3691,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>7</v>
@@ -3733,7 +3736,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Not Started")</f>
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>12</v>
@@ -3784,7 +3787,7 @@
       </c>
       <c r="E13">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A13,'Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F13">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A13,'Project Checklist'!$G$5:$G$220,"In Progress")</f>
@@ -3796,7 +3799,7 @@
       </c>
       <c r="H13" s="3">
         <f t="shared" ref="H13:H33" si="0">IF(D13=0,0,E13/D13)</f>
-        <v>0</v>
+        <v>0.6428571428571429</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -4586,7 +4589,7 @@
         <v>53</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>54</v>
@@ -4613,7 +4616,7 @@
         <v>57</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>54</v>
@@ -4640,7 +4643,7 @@
         <v>61</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>54</v>
@@ -4667,7 +4670,7 @@
         <v>64</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>54</v>
@@ -4694,7 +4697,7 @@
         <v>68</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>69</v>
@@ -4721,7 +4724,7 @@
         <v>73</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>54</v>
@@ -4748,7 +4751,7 @@
         <v>76</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>54</v>
@@ -4775,14 +4778,14 @@
         <v>79</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>54</v>
       </c>
       <c r="I12" s="18"/>
     </row>
-    <row r="13" spans="1:9" ht="28.3">
+    <row r="13" spans="1:9" ht="42.45">
       <c r="A13" s="15" t="s">
         <v>80</v>
       </c>
@@ -4802,12 +4805,14 @@
         <v>83</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="I13" s="18"/>
+      <c r="I13" s="18" t="s">
+        <v>932</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="28.3">
       <c r="A14" s="15" t="s">
@@ -11391,6 +11396,7 @@
     <mergeCell ref="A1:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
restructured folder, updated checklist
</commit_message>
<xml_diff>
--- a/NetLabz_Project_Checklist.xlsx
+++ b/NetLabz_Project_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NetLabz_Enterprise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E31B397-A22C-4E88-870D-36F7719DAE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27857B8C-BFE4-42B4-94CB-7FB6C0E6D873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="29692" windowHeight="11829" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="29692" windowHeight="11829" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1745" uniqueCount="853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1748" uniqueCount="856">
   <si>
     <t>Overall Progress</t>
   </si>
@@ -2595,6 +2595,15 @@
   </si>
   <si>
     <t>Used AI to list file types that are common with VM's so as not to miss any, creating vulnerability.</t>
+  </si>
+  <si>
+    <t>Created all my vswitches 1x External, 3x Internal</t>
+  </si>
+  <si>
+    <t>Would need to install wireshark inside VM to capture arp and icmp unicast replies. Currently only captures broadcasts.</t>
+  </si>
+  <si>
+    <t>No routing capabilities yet, so adding this section later.</t>
   </si>
 </sst>
 </file>
@@ -2915,54 +2924,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF2F5597"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF2F5597"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -3118,6 +3079,54 @@
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF2F5597"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF2F5597"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3132,7 +3141,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectChecklistTable" displayName="ProjectChecklistTable" ref="A4:I220" totalsRowShown="0" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectChecklistTable" displayName="ProjectChecklistTable" ref="A4:I220" totalsRowShown="0" dataDxfId="13">
   <autoFilter ref="A4:I220" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="6">
       <filters>
@@ -3141,15 +3150,15 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Task ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Phase #" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Phase" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Category" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Task" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Deliverable / Evidence" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Priority" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Notes" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Task ID" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Phase #" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Phase" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Category" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Task" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Deliverable / Evidence" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Priority" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Notes" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3170,7 +3179,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0DFA51D1-C4E7-4297-A332-2A07FE6908A6}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0DFA51D1-C4E7-4297-A332-2A07FE6908A6}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="15">
   <autoFilter ref="A1:C8" xr:uid="{0DFA51D1-C4E7-4297-A332-2A07FE6908A6}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{84782901-9C62-43D0-9F45-B6BDD25C78B2}" name="Network"/>
@@ -3182,7 +3191,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A49B7CAB-322A-4674-B078-48D9A820176E}" name="Table4" displayName="Table4" ref="A11:B18" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A49B7CAB-322A-4674-B078-48D9A820176E}" name="Table4" displayName="Table4" ref="A11:B18" totalsRowShown="0" headerRowDxfId="14">
   <autoFilter ref="A11:B18" xr:uid="{A49B7CAB-322A-4674-B078-48D9A820176E}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E986A977-7F13-4F5C-AB41-2E2F4CECF81A}" name="Address Range"/>
@@ -3427,7 +3436,7 @@
       </c>
       <c r="B4" s="4">
         <f>IF(B5=0,0,B6/B5)</f>
-        <v>6.9444444444444448E-2</v>
+        <v>8.7962962962962965E-2</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>1</v>
@@ -3457,7 +3466,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>7</v>
@@ -3487,7 +3496,7 @@
       </c>
       <c r="B8" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Blocked")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>6</v>
@@ -3502,7 +3511,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Not Started")</f>
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>12</v>
@@ -3584,7 +3593,7 @@
       </c>
       <c r="E14">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A14,'Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F14">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A14,'Project Checklist'!$G$5:$G$220,"In Progress")</f>
@@ -3592,11 +3601,11 @@
       </c>
       <c r="G14">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A14,'Project Checklist'!$G$5:$G$220,"Blocked")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14" s="3">
         <f t="shared" si="0"/>
-        <v>0.1111111111111111</v>
+        <v>0.55555555555555558</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4742,7 +4751,7 @@
       </c>
       <c r="I19" s="16"/>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" ht="28.3">
       <c r="A20" s="13" t="s">
         <v>105</v>
       </c>
@@ -4762,12 +4771,14 @@
         <v>107</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="I20" s="16"/>
+      <c r="I20" s="16" t="s">
+        <v>853</v>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="28.3">
       <c r="A21" s="13" t="s">
@@ -4789,7 +4800,7 @@
         <v>111</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>54</v>
@@ -4816,7 +4827,7 @@
         <v>115</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>54</v>
@@ -4843,14 +4854,14 @@
         <v>119</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>54</v>
       </c>
       <c r="I23" s="16"/>
     </row>
-    <row r="24" spans="1:9" ht="28.3">
+    <row r="24" spans="1:9" ht="42.45">
       <c r="A24" s="13" t="s">
         <v>120</v>
       </c>
@@ -4870,12 +4881,14 @@
         <v>123</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="I24" s="16"/>
+      <c r="I24" s="16" t="s">
+        <v>854</v>
+      </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="13" t="s">
@@ -4897,7 +4910,7 @@
         <v>126</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>69</v>
@@ -4924,12 +4937,14 @@
         <v>130</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="I26" s="16"/>
+      <c r="I26" s="16" t="s">
+        <v>855</v>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="28.3">
       <c r="A27" s="13" t="s">

</xml_diff>

<commit_message>
updated phase 1 README, updaated checklist
</commit_message>
<xml_diff>
--- a/NetLabz_Project_Checklist.xlsx
+++ b/NetLabz_Project_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NetLabz_Enterprise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27857B8C-BFE4-42B4-94CB-7FB6C0E6D873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD08026-734A-4D80-B372-7F2F43914BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="29692" windowHeight="11829" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2924,6 +2924,54 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF2F5597"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF2F5597"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -3079,54 +3127,6 @@
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF2F5597"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF2F5597"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3141,24 +3141,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectChecklistTable" displayName="ProjectChecklistTable" ref="A4:I220" totalsRowShown="0" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectChecklistTable" displayName="ProjectChecklistTable" ref="A4:I220" totalsRowShown="0" dataDxfId="15">
   <autoFilter ref="A4:I220" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="6">
       <filters>
+        <filter val="Blocked"/>
         <filter val="Not Started"/>
+        <filter val="Skipped"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Task ID" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Phase #" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Phase" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Category" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Task" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Deliverable / Evidence" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Priority" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Notes" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Task ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Phase #" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Phase" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Category" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Task" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Deliverable / Evidence" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Priority" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Notes" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3179,7 +3181,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0DFA51D1-C4E7-4297-A332-2A07FE6908A6}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0DFA51D1-C4E7-4297-A332-2A07FE6908A6}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:C8" xr:uid="{0DFA51D1-C4E7-4297-A332-2A07FE6908A6}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{84782901-9C62-43D0-9F45-B6BDD25C78B2}" name="Network"/>
@@ -3191,7 +3193,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A49B7CAB-322A-4674-B078-48D9A820176E}" name="Table4" displayName="Table4" ref="A11:B18" totalsRowShown="0" headerRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A49B7CAB-322A-4674-B078-48D9A820176E}" name="Table4" displayName="Table4" ref="A11:B18" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A11:B18" xr:uid="{A49B7CAB-322A-4674-B078-48D9A820176E}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E986A977-7F13-4F5C-AB41-2E2F4CECF81A}" name="Address Range"/>
@@ -3436,7 +3438,7 @@
       </c>
       <c r="B4" s="4">
         <f>IF(B5=0,0,B6/B5)</f>
-        <v>8.7962962962962965E-2</v>
+        <v>9.2592592592592587E-2</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>1</v>
@@ -3466,7 +3468,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>7</v>
@@ -3511,7 +3513,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Not Started")</f>
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>12</v>
@@ -3593,7 +3595,7 @@
       </c>
       <c r="E14">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A14,'Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A14,'Project Checklist'!$G$5:$G$220,"In Progress")</f>
@@ -3605,7 +3607,7 @@
       </c>
       <c r="H14" s="3">
         <f t="shared" si="0"/>
-        <v>0.55555555555555558</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4751,7 +4753,7 @@
       </c>
       <c r="I19" s="16"/>
     </row>
-    <row r="20" spans="1:9" ht="28.3">
+    <row r="20" spans="1:9" ht="28.3" hidden="1">
       <c r="A20" s="13" t="s">
         <v>105</v>
       </c>
@@ -4780,7 +4782,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="28.3">
+    <row r="21" spans="1:9" ht="28.3" hidden="1">
       <c r="A21" s="13" t="s">
         <v>108</v>
       </c>
@@ -4807,7 +4809,7 @@
       </c>
       <c r="I21" s="16"/>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" hidden="1">
       <c r="A22" s="13" t="s">
         <v>112</v>
       </c>
@@ -4834,7 +4836,7 @@
       </c>
       <c r="I22" s="16"/>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" hidden="1">
       <c r="A23" s="13" t="s">
         <v>116</v>
       </c>
@@ -4946,7 +4948,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="28.3">
+    <row r="27" spans="1:9" ht="28.3" hidden="1">
       <c r="A27" s="13" t="s">
         <v>131</v>
       </c>
@@ -4966,7 +4968,7 @@
         <v>133</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
updating next steps on main README
</commit_message>
<xml_diff>
--- a/NetLabz_Project_Checklist.xlsx
+++ b/NetLabz_Project_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NetLabz_Enterprise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD08026-734A-4D80-B372-7F2F43914BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90AF1A87-C505-4236-905B-8E7348B61BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="29692" windowHeight="11829" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1748" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="857">
   <si>
     <t>Overall Progress</t>
   </si>
@@ -2604,6 +2604,9 @@
   </si>
   <si>
     <t>No routing capabilities yet, so adding this section later.</t>
+  </si>
+  <si>
+    <t>Selecting OPNSense</t>
   </si>
 </sst>
 </file>
@@ -3483,7 +3486,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"In Progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>9</v>
@@ -3513,7 +3516,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Not Started")</f>
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>12</v>
@@ -3630,7 +3633,7 @@
       </c>
       <c r="F15">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A15,'Project Checklist'!$G$5:$G$220,"In Progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A15,'Project Checklist'!$G$5:$G$220,"Blocked")</f>
@@ -4975,7 +4978,7 @@
       </c>
       <c r="I27" s="16"/>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" ht="28.3">
       <c r="A28" s="13" t="s">
         <v>134</v>
       </c>
@@ -4995,12 +4998,14 @@
         <v>137</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="I28" s="16"/>
+      <c r="I28" s="16" t="s">
+        <v>856</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="28.3">
       <c r="A29" s="13" t="s">

</xml_diff>

<commit_message>
P02-09 process and documentation, screenshots
</commit_message>
<xml_diff>
--- a/NetLabz_Project_Checklist.xlsx
+++ b/NetLabz_Project_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NetLabz_Enterprise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BD4489-8C13-4EF9-B492-48F44840843F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36C65DA-6DEF-4765-8000-3E18F316CE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="29692" windowHeight="11829" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B4" s="4">
         <f>IF(B5=0,0,B6/B5)</f>
-        <v>0.11574074074074074</v>
+        <v>0.12962962962962962</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>1</v>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>7</v>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Project Checklist'!$G$5:$G$220,"Not Started")</f>
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>12</v>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="E15">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A15,'Project Checklist'!$G$5:$G$220,"Complete")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F15">
         <f>COUNTIFS('Project Checklist'!$B$5:$B$220,A15,'Project Checklist'!$G$5:$G$220,"In Progress")</f>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H15" s="3">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="I27" s="16"/>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" hidden="1">
       <c r="A28" s="13" t="s">
         <v>134</v>
       </c>
@@ -5007,7 +5007,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="28.3">
+    <row r="29" spans="1:9" ht="28.3" hidden="1">
       <c r="A29" s="13" t="s">
         <v>138</v>
       </c>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="I29" s="16"/>
     </row>
-    <row r="30" spans="1:9" ht="28.3">
+    <row r="30" spans="1:9" ht="28.3" hidden="1">
       <c r="A30" s="13" t="s">
         <v>141</v>
       </c>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="I30" s="16"/>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" hidden="1">
       <c r="A31" s="13" t="s">
         <v>144</v>
       </c>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="I31" s="16"/>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" hidden="1">
       <c r="A32" s="13" t="s">
         <v>147</v>
       </c>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="I32" s="16"/>
     </row>
-    <row r="33" spans="1:9" ht="28.3">
+    <row r="33" spans="1:9" ht="28.3" hidden="1">
       <c r="A33" s="13" t="s">
         <v>151</v>
       </c>
@@ -5135,14 +5135,14 @@
         <v>154</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H33" s="15" t="s">
         <v>54</v>
       </c>
       <c r="I33" s="16"/>
     </row>
-    <row r="34" spans="1:9" ht="28.3">
+    <row r="34" spans="1:9" ht="28.3" hidden="1">
       <c r="A34" s="13" t="s">
         <v>155</v>
       </c>
@@ -5162,14 +5162,14 @@
         <v>157</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H34" s="15" t="s">
         <v>54</v>
       </c>
       <c r="I34" s="16"/>
     </row>
-    <row r="35" spans="1:9" ht="28.3">
+    <row r="35" spans="1:9" ht="28.3" hidden="1">
       <c r="A35" s="13" t="s">
         <v>158</v>
       </c>
@@ -5189,7 +5189,7 @@
         <v>160</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H35" s="15" t="s">
         <v>54</v>

</xml_diff>